<commit_message>
Estados añadidos y logica rapida de solicitudes a sumarios
</commit_message>
<xml_diff>
--- a/storage/app/templates/FORMATO SALIDA MATERIAL.xlsx
+++ b/storage/app/templates/FORMATO SALIDA MATERIAL.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\laragon\www\SISTEMA-OFICIAL-AGARCORP\storage\app\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{66B6A30F-440E-40D7-891B-7D7B8CDFE4A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F94A1411-F154-414B-98E4-BE2026FA26FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="22932" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{A5D087B2-5B39-4E10-8501-AE53E41EA51F}"/>
   </bookViews>
@@ -303,7 +303,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="38">
+  <cellXfs count="39">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
@@ -324,95 +324,98 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="2" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="2" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="2" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="2" fillId="0" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="2" fillId="0" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="5" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="5" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="2" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="2" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="2" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="2" fillId="0" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="2" fillId="0" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -839,184 +842,184 @@
     <row r="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1" s="7"/>
       <c r="B1" s="7"/>
-      <c r="C1" s="8" t="s">
+      <c r="C1" s="35" t="s">
         <v>0</v>
       </c>
-      <c r="D1" s="8"/>
-      <c r="E1" s="8"/>
-      <c r="F1" s="8"/>
-      <c r="G1" s="8"/>
-      <c r="H1" s="8"/>
-      <c r="I1" s="8"/>
-      <c r="J1" s="8"/>
-      <c r="K1" s="8"/>
-      <c r="L1" s="9" t="s">
+      <c r="D1" s="35"/>
+      <c r="E1" s="35"/>
+      <c r="F1" s="35"/>
+      <c r="G1" s="35"/>
+      <c r="H1" s="35"/>
+      <c r="I1" s="35"/>
+      <c r="J1" s="35"/>
+      <c r="K1" s="35"/>
+      <c r="L1" s="21" t="s">
         <v>1</v>
       </c>
-      <c r="M1" s="9"/>
-      <c r="N1" s="9"/>
+      <c r="M1" s="21"/>
+      <c r="N1" s="21"/>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A2" s="7"/>
       <c r="B2" s="7"/>
-      <c r="C2" s="8"/>
-      <c r="D2" s="8"/>
-      <c r="E2" s="8"/>
-      <c r="F2" s="8"/>
-      <c r="G2" s="8"/>
-      <c r="H2" s="8"/>
-      <c r="I2" s="8"/>
-      <c r="J2" s="8"/>
-      <c r="K2" s="8"/>
-      <c r="L2" s="10" t="s">
+      <c r="C2" s="35"/>
+      <c r="D2" s="35"/>
+      <c r="E2" s="35"/>
+      <c r="F2" s="35"/>
+      <c r="G2" s="35"/>
+      <c r="H2" s="35"/>
+      <c r="I2" s="35"/>
+      <c r="J2" s="35"/>
+      <c r="K2" s="35"/>
+      <c r="L2" s="36" t="s">
         <v>2</v>
       </c>
-      <c r="M2" s="10"/>
-      <c r="N2" s="10"/>
+      <c r="M2" s="36"/>
+      <c r="N2" s="36"/>
     </row>
     <row r="3" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A3" s="7"/>
       <c r="B3" s="7"/>
-      <c r="C3" s="8"/>
-      <c r="D3" s="8"/>
-      <c r="E3" s="8"/>
-      <c r="F3" s="8"/>
-      <c r="G3" s="8"/>
-      <c r="H3" s="8"/>
-      <c r="I3" s="8"/>
-      <c r="J3" s="8"/>
-      <c r="K3" s="8"/>
-      <c r="L3" s="10" t="s">
+      <c r="C3" s="35"/>
+      <c r="D3" s="35"/>
+      <c r="E3" s="35"/>
+      <c r="F3" s="35"/>
+      <c r="G3" s="35"/>
+      <c r="H3" s="35"/>
+      <c r="I3" s="35"/>
+      <c r="J3" s="35"/>
+      <c r="K3" s="35"/>
+      <c r="L3" s="36" t="s">
         <v>3</v>
       </c>
-      <c r="M3" s="10"/>
-      <c r="N3" s="10"/>
+      <c r="M3" s="36"/>
+      <c r="N3" s="36"/>
     </row>
     <row r="4" spans="1:14" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="7"/>
       <c r="B4" s="7"/>
-      <c r="C4" s="8"/>
-      <c r="D4" s="8"/>
-      <c r="E4" s="8"/>
-      <c r="F4" s="8"/>
-      <c r="G4" s="8"/>
-      <c r="H4" s="8"/>
-      <c r="I4" s="8"/>
-      <c r="J4" s="8"/>
-      <c r="K4" s="8"/>
-      <c r="L4" s="11" t="s">
+      <c r="C4" s="35"/>
+      <c r="D4" s="35"/>
+      <c r="E4" s="35"/>
+      <c r="F4" s="35"/>
+      <c r="G4" s="35"/>
+      <c r="H4" s="35"/>
+      <c r="I4" s="35"/>
+      <c r="J4" s="35"/>
+      <c r="K4" s="35"/>
+      <c r="L4" s="37" t="s">
         <v>4</v>
       </c>
-      <c r="M4" s="11"/>
-      <c r="N4" s="11"/>
+      <c r="M4" s="37"/>
+      <c r="N4" s="37"/>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A5" s="14" t="s">
+      <c r="A5" s="20" t="s">
         <v>5</v>
       </c>
-      <c r="B5" s="14"/>
-      <c r="C5" s="14"/>
-      <c r="D5" s="14"/>
-      <c r="E5" s="14"/>
-      <c r="F5" s="14" t="s">
+      <c r="B5" s="20"/>
+      <c r="C5" s="20"/>
+      <c r="D5" s="20"/>
+      <c r="E5" s="20"/>
+      <c r="F5" s="20" t="s">
         <v>6</v>
       </c>
-      <c r="G5" s="14"/>
-      <c r="H5" s="14"/>
-      <c r="I5" s="14"/>
-      <c r="J5" s="14"/>
-      <c r="K5" s="14"/>
-      <c r="L5" s="15"/>
-      <c r="M5" s="13"/>
-      <c r="N5" s="13"/>
+      <c r="G5" s="20"/>
+      <c r="H5" s="20"/>
+      <c r="I5" s="20"/>
+      <c r="J5" s="20"/>
+      <c r="K5" s="20"/>
+      <c r="L5" s="33"/>
+      <c r="M5" s="34"/>
+      <c r="N5" s="34"/>
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A6" s="14" t="s">
+      <c r="A6" s="20" t="s">
         <v>8</v>
       </c>
-      <c r="B6" s="14"/>
-      <c r="C6" s="14"/>
-      <c r="D6" s="14"/>
-      <c r="E6" s="14"/>
-      <c r="F6" s="14"/>
-      <c r="G6" s="14"/>
-      <c r="H6" s="14"/>
-      <c r="I6" s="14"/>
-      <c r="J6" s="14" t="s">
+      <c r="B6" s="20"/>
+      <c r="C6" s="20"/>
+      <c r="D6" s="20"/>
+      <c r="E6" s="20"/>
+      <c r="F6" s="20"/>
+      <c r="G6" s="20"/>
+      <c r="H6" s="20"/>
+      <c r="I6" s="20"/>
+      <c r="J6" s="20" t="s">
         <v>9</v>
       </c>
-      <c r="K6" s="14"/>
-      <c r="L6" s="14"/>
-      <c r="M6" s="14"/>
-      <c r="N6" s="14"/>
+      <c r="K6" s="20"/>
+      <c r="L6" s="20"/>
+      <c r="M6" s="20"/>
+      <c r="N6" s="20"/>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A7" s="12" t="s">
+      <c r="A7" s="32" t="s">
         <v>10</v>
       </c>
-      <c r="B7" s="13" t="s">
+      <c r="B7" s="34" t="s">
         <v>11</v>
       </c>
-      <c r="C7" s="13"/>
-      <c r="D7" s="13"/>
-      <c r="E7" s="13"/>
-      <c r="F7" s="13"/>
-      <c r="G7" s="12" t="s">
+      <c r="C7" s="34"/>
+      <c r="D7" s="34"/>
+      <c r="E7" s="34"/>
+      <c r="F7" s="34"/>
+      <c r="G7" s="32" t="s">
         <v>12</v>
       </c>
-      <c r="H7" s="12"/>
-      <c r="I7" s="12"/>
-      <c r="J7" s="12" t="s">
+      <c r="H7" s="32"/>
+      <c r="I7" s="32"/>
+      <c r="J7" s="32" t="s">
         <v>13</v>
       </c>
-      <c r="K7" s="12" t="s">
+      <c r="K7" s="32" t="s">
         <v>14</v>
       </c>
-      <c r="L7" s="12"/>
-      <c r="M7" s="12" t="s">
+      <c r="L7" s="32"/>
+      <c r="M7" s="32" t="s">
         <v>15</v>
       </c>
-      <c r="N7" s="12"/>
+      <c r="N7" s="32"/>
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A8" s="12"/>
-      <c r="B8" s="13"/>
-      <c r="C8" s="13"/>
-      <c r="D8" s="13"/>
-      <c r="E8" s="13"/>
-      <c r="F8" s="13"/>
-      <c r="G8" s="12" t="s">
+      <c r="A8" s="32"/>
+      <c r="B8" s="34"/>
+      <c r="C8" s="34"/>
+      <c r="D8" s="34"/>
+      <c r="E8" s="34"/>
+      <c r="F8" s="34"/>
+      <c r="G8" s="32" t="s">
         <v>16</v>
       </c>
-      <c r="H8" s="12"/>
+      <c r="H8" s="32"/>
       <c r="I8" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="J8" s="12"/>
+      <c r="J8" s="32"/>
       <c r="K8" s="3" t="s">
         <v>18</v>
       </c>
       <c r="L8" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="M8" s="12"/>
-      <c r="N8" s="12"/>
+      <c r="M8" s="32"/>
+      <c r="N8" s="32"/>
     </row>
     <row r="9" spans="1:14" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="B9" s="16" t="s">
+      <c r="B9" s="29" t="s">
         <v>32</v>
       </c>
-      <c r="C9" s="16"/>
-      <c r="D9" s="16"/>
-      <c r="E9" s="16"/>
-      <c r="F9" s="17"/>
-      <c r="G9" s="18" t="s">
+      <c r="C9" s="29"/>
+      <c r="D9" s="29"/>
+      <c r="E9" s="29"/>
+      <c r="F9" s="30"/>
+      <c r="G9" s="31" t="s">
         <v>35</v>
       </c>
-      <c r="H9" s="17"/>
+      <c r="H9" s="30"/>
       <c r="I9" s="2" t="str">
         <f>IFERROR((_xlfn.XLOOKUP(#REF!,#REF!,#REF!))," " )</f>
         <v xml:space="preserve"> </v>
@@ -1024,32 +1027,32 @@
       <c r="J9" s="6" t="s">
         <v>33</v>
       </c>
-      <c r="K9" s="6" t="s">
+      <c r="K9" s="38" t="s">
         <v>36</v>
       </c>
-      <c r="L9" s="6" t="s">
+      <c r="L9" s="38" t="s">
         <v>37</v>
       </c>
-      <c r="M9" s="18" t="s">
+      <c r="M9" s="31" t="s">
         <v>38</v>
       </c>
-      <c r="N9" s="17"/>
+      <c r="N9" s="30"/>
     </row>
     <row r="10" spans="1:14" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="B10" s="16" t="s">
+      <c r="B10" s="29" t="s">
         <v>32</v>
       </c>
-      <c r="C10" s="16"/>
-      <c r="D10" s="16"/>
-      <c r="E10" s="16"/>
-      <c r="F10" s="17"/>
-      <c r="G10" s="18" t="s">
+      <c r="C10" s="29"/>
+      <c r="D10" s="29"/>
+      <c r="E10" s="29"/>
+      <c r="F10" s="30"/>
+      <c r="G10" s="31" t="s">
         <v>35</v>
       </c>
-      <c r="H10" s="17"/>
+      <c r="H10" s="30"/>
       <c r="I10" s="2" t="str">
         <f>IFERROR((_xlfn.XLOOKUP(#REF!,#REF!,#REF!))," " )</f>
         <v xml:space="preserve"> </v>
@@ -1057,32 +1060,32 @@
       <c r="J10" s="6" t="s">
         <v>33</v>
       </c>
-      <c r="K10" s="6" t="s">
+      <c r="K10" s="38" t="s">
         <v>36</v>
       </c>
-      <c r="L10" s="6" t="s">
+      <c r="L10" s="38" t="s">
         <v>37</v>
       </c>
-      <c r="M10" s="18" t="s">
+      <c r="M10" s="31" t="s">
         <v>38</v>
       </c>
-      <c r="N10" s="17"/>
+      <c r="N10" s="30"/>
     </row>
     <row r="11" spans="1:14" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="B11" s="16" t="s">
+      <c r="B11" s="29" t="s">
         <v>32</v>
       </c>
-      <c r="C11" s="16"/>
-      <c r="D11" s="16"/>
-      <c r="E11" s="16"/>
-      <c r="F11" s="17"/>
-      <c r="G11" s="18" t="s">
+      <c r="C11" s="29"/>
+      <c r="D11" s="29"/>
+      <c r="E11" s="29"/>
+      <c r="F11" s="30"/>
+      <c r="G11" s="31" t="s">
         <v>35</v>
       </c>
-      <c r="H11" s="17"/>
+      <c r="H11" s="30"/>
       <c r="I11" s="2" t="str">
         <f>IFERROR((_xlfn.XLOOKUP(#REF!,#REF!,#REF!))," " )</f>
         <v xml:space="preserve"> </v>
@@ -1090,32 +1093,32 @@
       <c r="J11" s="6" t="s">
         <v>33</v>
       </c>
-      <c r="K11" s="6" t="s">
+      <c r="K11" s="38" t="s">
         <v>36</v>
       </c>
-      <c r="L11" s="6" t="s">
+      <c r="L11" s="38" t="s">
         <v>37</v>
       </c>
-      <c r="M11" s="18" t="s">
+      <c r="M11" s="31" t="s">
         <v>38</v>
       </c>
-      <c r="N11" s="17"/>
+      <c r="N11" s="30"/>
     </row>
     <row r="12" spans="1:14" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="B12" s="16" t="s">
+      <c r="B12" s="29" t="s">
         <v>32</v>
       </c>
-      <c r="C12" s="16"/>
-      <c r="D12" s="16"/>
-      <c r="E12" s="16"/>
-      <c r="F12" s="17"/>
-      <c r="G12" s="18" t="s">
+      <c r="C12" s="29"/>
+      <c r="D12" s="29"/>
+      <c r="E12" s="29"/>
+      <c r="F12" s="30"/>
+      <c r="G12" s="31" t="s">
         <v>35</v>
       </c>
-      <c r="H12" s="17"/>
+      <c r="H12" s="30"/>
       <c r="I12" s="2" t="str">
         <f>IFERROR((_xlfn.XLOOKUP(#REF!,#REF!,#REF!))," " )</f>
         <v xml:space="preserve"> </v>
@@ -1123,32 +1126,32 @@
       <c r="J12" s="6" t="s">
         <v>33</v>
       </c>
-      <c r="K12" s="6" t="s">
+      <c r="K12" s="38" t="s">
         <v>36</v>
       </c>
-      <c r="L12" s="6" t="s">
+      <c r="L12" s="38" t="s">
         <v>37</v>
       </c>
-      <c r="M12" s="18" t="s">
+      <c r="M12" s="31" t="s">
         <v>38</v>
       </c>
-      <c r="N12" s="17"/>
+      <c r="N12" s="30"/>
     </row>
     <row r="13" spans="1:14" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="B13" s="16" t="s">
+      <c r="B13" s="29" t="s">
         <v>32</v>
       </c>
-      <c r="C13" s="16"/>
-      <c r="D13" s="16"/>
-      <c r="E13" s="16"/>
-      <c r="F13" s="17"/>
-      <c r="G13" s="18" t="s">
+      <c r="C13" s="29"/>
+      <c r="D13" s="29"/>
+      <c r="E13" s="29"/>
+      <c r="F13" s="30"/>
+      <c r="G13" s="31" t="s">
         <v>35</v>
       </c>
-      <c r="H13" s="17"/>
+      <c r="H13" s="30"/>
       <c r="I13" s="2" t="str">
         <f>IFERROR((_xlfn.XLOOKUP(#REF!,#REF!,#REF!))," " )</f>
         <v xml:space="preserve"> </v>
@@ -1156,32 +1159,32 @@
       <c r="J13" s="6" t="s">
         <v>33</v>
       </c>
-      <c r="K13" s="6" t="s">
+      <c r="K13" s="38" t="s">
         <v>36</v>
       </c>
-      <c r="L13" s="6" t="s">
+      <c r="L13" s="38" t="s">
         <v>37</v>
       </c>
-      <c r="M13" s="18" t="s">
+      <c r="M13" s="31" t="s">
         <v>38</v>
       </c>
-      <c r="N13" s="17"/>
+      <c r="N13" s="30"/>
     </row>
     <row r="14" spans="1:14" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="B14" s="16" t="s">
+      <c r="B14" s="29" t="s">
         <v>32</v>
       </c>
-      <c r="C14" s="16"/>
-      <c r="D14" s="16"/>
-      <c r="E14" s="16"/>
-      <c r="F14" s="17"/>
-      <c r="G14" s="18" t="s">
+      <c r="C14" s="29"/>
+      <c r="D14" s="29"/>
+      <c r="E14" s="29"/>
+      <c r="F14" s="30"/>
+      <c r="G14" s="31" t="s">
         <v>35</v>
       </c>
-      <c r="H14" s="17"/>
+      <c r="H14" s="30"/>
       <c r="I14" s="2" t="str">
         <f>IFERROR((_xlfn.XLOOKUP(#REF!,#REF!,#REF!))," " )</f>
         <v xml:space="preserve"> </v>
@@ -1189,32 +1192,32 @@
       <c r="J14" s="6" t="s">
         <v>33</v>
       </c>
-      <c r="K14" s="6" t="s">
+      <c r="K14" s="38" t="s">
         <v>36</v>
       </c>
-      <c r="L14" s="6" t="s">
+      <c r="L14" s="38" t="s">
         <v>37</v>
       </c>
-      <c r="M14" s="18" t="s">
+      <c r="M14" s="31" t="s">
         <v>38</v>
       </c>
-      <c r="N14" s="17"/>
+      <c r="N14" s="30"/>
     </row>
     <row r="15" spans="1:14" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="B15" s="16" t="s">
+      <c r="B15" s="29" t="s">
         <v>32</v>
       </c>
-      <c r="C15" s="16"/>
-      <c r="D15" s="16"/>
-      <c r="E15" s="16"/>
-      <c r="F15" s="17"/>
-      <c r="G15" s="18" t="s">
+      <c r="C15" s="29"/>
+      <c r="D15" s="29"/>
+      <c r="E15" s="29"/>
+      <c r="F15" s="30"/>
+      <c r="G15" s="31" t="s">
         <v>35</v>
       </c>
-      <c r="H15" s="17"/>
+      <c r="H15" s="30"/>
       <c r="I15" s="2" t="str">
         <f>IFERROR((_xlfn.XLOOKUP(#REF!,#REF!,#REF!))," " )</f>
         <v xml:space="preserve"> </v>
@@ -1222,32 +1225,32 @@
       <c r="J15" s="6" t="s">
         <v>33</v>
       </c>
-      <c r="K15" s="6" t="s">
+      <c r="K15" s="38" t="s">
         <v>36</v>
       </c>
-      <c r="L15" s="6" t="s">
+      <c r="L15" s="38" t="s">
         <v>37</v>
       </c>
-      <c r="M15" s="18" t="s">
+      <c r="M15" s="31" t="s">
         <v>38</v>
       </c>
-      <c r="N15" s="17"/>
+      <c r="N15" s="30"/>
     </row>
     <row r="16" spans="1:14" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="B16" s="16" t="s">
+      <c r="B16" s="29" t="s">
         <v>32</v>
       </c>
-      <c r="C16" s="16"/>
-      <c r="D16" s="16"/>
-      <c r="E16" s="16"/>
-      <c r="F16" s="17"/>
-      <c r="G16" s="18" t="s">
+      <c r="C16" s="29"/>
+      <c r="D16" s="29"/>
+      <c r="E16" s="29"/>
+      <c r="F16" s="30"/>
+      <c r="G16" s="31" t="s">
         <v>35</v>
       </c>
-      <c r="H16" s="17"/>
+      <c r="H16" s="30"/>
       <c r="I16" s="2" t="str">
         <f>IFERROR((_xlfn.XLOOKUP(#REF!,#REF!,#REF!))," " )</f>
         <v xml:space="preserve"> </v>
@@ -1255,32 +1258,32 @@
       <c r="J16" s="6" t="s">
         <v>33</v>
       </c>
-      <c r="K16" s="6" t="s">
+      <c r="K16" s="38" t="s">
         <v>36</v>
       </c>
-      <c r="L16" s="6" t="s">
+      <c r="L16" s="38" t="s">
         <v>37</v>
       </c>
-      <c r="M16" s="18" t="s">
+      <c r="M16" s="31" t="s">
         <v>38</v>
       </c>
-      <c r="N16" s="17"/>
+      <c r="N16" s="30"/>
     </row>
     <row r="17" spans="1:14" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="B17" s="16" t="s">
+      <c r="B17" s="29" t="s">
         <v>32</v>
       </c>
-      <c r="C17" s="16"/>
-      <c r="D17" s="16"/>
-      <c r="E17" s="16"/>
-      <c r="F17" s="17"/>
-      <c r="G17" s="18" t="s">
+      <c r="C17" s="29"/>
+      <c r="D17" s="29"/>
+      <c r="E17" s="29"/>
+      <c r="F17" s="30"/>
+      <c r="G17" s="31" t="s">
         <v>35</v>
       </c>
-      <c r="H17" s="17"/>
+      <c r="H17" s="30"/>
       <c r="I17" s="2" t="str">
         <f>IFERROR((_xlfn.XLOOKUP(#REF!,#REF!,#REF!))," " )</f>
         <v xml:space="preserve"> </v>
@@ -1288,32 +1291,32 @@
       <c r="J17" s="6" t="s">
         <v>33</v>
       </c>
-      <c r="K17" s="6" t="s">
+      <c r="K17" s="38" t="s">
         <v>36</v>
       </c>
-      <c r="L17" s="6" t="s">
+      <c r="L17" s="38" t="s">
         <v>37</v>
       </c>
-      <c r="M17" s="18" t="s">
+      <c r="M17" s="31" t="s">
         <v>38</v>
       </c>
-      <c r="N17" s="17"/>
+      <c r="N17" s="30"/>
     </row>
     <row r="18" spans="1:14" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="B18" s="16" t="s">
+      <c r="B18" s="29" t="s">
         <v>32</v>
       </c>
-      <c r="C18" s="16"/>
-      <c r="D18" s="16"/>
-      <c r="E18" s="16"/>
-      <c r="F18" s="17"/>
-      <c r="G18" s="18" t="s">
+      <c r="C18" s="29"/>
+      <c r="D18" s="29"/>
+      <c r="E18" s="29"/>
+      <c r="F18" s="30"/>
+      <c r="G18" s="31" t="s">
         <v>35</v>
       </c>
-      <c r="H18" s="17"/>
+      <c r="H18" s="30"/>
       <c r="I18" s="2" t="str">
         <f>IFERROR((_xlfn.XLOOKUP(#REF!,#REF!,#REF!))," " )</f>
         <v xml:space="preserve"> </v>
@@ -1321,32 +1324,32 @@
       <c r="J18" s="6" t="s">
         <v>33</v>
       </c>
-      <c r="K18" s="6" t="s">
+      <c r="K18" s="38" t="s">
         <v>36</v>
       </c>
-      <c r="L18" s="6" t="s">
+      <c r="L18" s="38" t="s">
         <v>37</v>
       </c>
-      <c r="M18" s="18" t="s">
+      <c r="M18" s="31" t="s">
         <v>38</v>
       </c>
-      <c r="N18" s="17"/>
+      <c r="N18" s="30"/>
     </row>
     <row r="19" spans="1:14" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="B19" s="16" t="s">
+      <c r="B19" s="29" t="s">
         <v>32</v>
       </c>
-      <c r="C19" s="16"/>
-      <c r="D19" s="16"/>
-      <c r="E19" s="16"/>
-      <c r="F19" s="17"/>
-      <c r="G19" s="18" t="s">
+      <c r="C19" s="29"/>
+      <c r="D19" s="29"/>
+      <c r="E19" s="29"/>
+      <c r="F19" s="30"/>
+      <c r="G19" s="31" t="s">
         <v>35</v>
       </c>
-      <c r="H19" s="17"/>
+      <c r="H19" s="30"/>
       <c r="I19" s="2" t="str">
         <f>IFERROR((_xlfn.XLOOKUP(#REF!,#REF!,#REF!))," " )</f>
         <v xml:space="preserve"> </v>
@@ -1354,32 +1357,32 @@
       <c r="J19" s="6" t="s">
         <v>33</v>
       </c>
-      <c r="K19" s="6" t="s">
+      <c r="K19" s="38" t="s">
         <v>36</v>
       </c>
-      <c r="L19" s="6" t="s">
+      <c r="L19" s="38" t="s">
         <v>37</v>
       </c>
-      <c r="M19" s="18" t="s">
+      <c r="M19" s="31" t="s">
         <v>38</v>
       </c>
-      <c r="N19" s="17"/>
+      <c r="N19" s="30"/>
     </row>
     <row r="20" spans="1:14" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="B20" s="16" t="s">
+      <c r="B20" s="29" t="s">
         <v>32</v>
       </c>
-      <c r="C20" s="16"/>
-      <c r="D20" s="16"/>
-      <c r="E20" s="16"/>
-      <c r="F20" s="17"/>
-      <c r="G20" s="18" t="s">
+      <c r="C20" s="29"/>
+      <c r="D20" s="29"/>
+      <c r="E20" s="29"/>
+      <c r="F20" s="30"/>
+      <c r="G20" s="31" t="s">
         <v>35</v>
       </c>
-      <c r="H20" s="17"/>
+      <c r="H20" s="30"/>
       <c r="I20" s="2" t="str">
         <f>IFERROR((_xlfn.XLOOKUP(#REF!,#REF!,#REF!))," " )</f>
         <v xml:space="preserve"> </v>
@@ -1387,32 +1390,32 @@
       <c r="J20" s="6" t="s">
         <v>33</v>
       </c>
-      <c r="K20" s="6" t="s">
+      <c r="K20" s="38" t="s">
         <v>36</v>
       </c>
-      <c r="L20" s="6" t="s">
+      <c r="L20" s="38" t="s">
         <v>37</v>
       </c>
-      <c r="M20" s="18" t="s">
+      <c r="M20" s="31" t="s">
         <v>38</v>
       </c>
-      <c r="N20" s="17"/>
+      <c r="N20" s="30"/>
     </row>
     <row r="21" spans="1:14" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="B21" s="16" t="s">
+      <c r="B21" s="29" t="s">
         <v>32</v>
       </c>
-      <c r="C21" s="16"/>
-      <c r="D21" s="16"/>
-      <c r="E21" s="16"/>
-      <c r="F21" s="17"/>
-      <c r="G21" s="18" t="s">
+      <c r="C21" s="29"/>
+      <c r="D21" s="29"/>
+      <c r="E21" s="29"/>
+      <c r="F21" s="30"/>
+      <c r="G21" s="31" t="s">
         <v>35</v>
       </c>
-      <c r="H21" s="17"/>
+      <c r="H21" s="30"/>
       <c r="I21" s="2" t="str">
         <f>IFERROR((_xlfn.XLOOKUP(#REF!,#REF!,#REF!))," " )</f>
         <v xml:space="preserve"> </v>
@@ -1420,64 +1423,64 @@
       <c r="J21" s="6" t="s">
         <v>33</v>
       </c>
-      <c r="K21" s="6" t="s">
+      <c r="K21" s="38" t="s">
         <v>36</v>
       </c>
-      <c r="L21" s="6" t="s">
+      <c r="L21" s="38" t="s">
         <v>37</v>
       </c>
-      <c r="M21" s="18" t="s">
+      <c r="M21" s="31" t="s">
         <v>38</v>
       </c>
-      <c r="N21" s="17"/>
+      <c r="N21" s="30"/>
     </row>
     <row r="22" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A22" s="9" t="s">
+      <c r="A22" s="21" t="s">
         <v>20</v>
       </c>
-      <c r="B22" s="9"/>
-      <c r="C22" s="9"/>
-      <c r="D22" s="9"/>
-      <c r="E22" s="9"/>
-      <c r="F22" s="9"/>
-      <c r="G22" s="9"/>
-      <c r="H22" s="9" t="s">
+      <c r="B22" s="21"/>
+      <c r="C22" s="21"/>
+      <c r="D22" s="21"/>
+      <c r="E22" s="21"/>
+      <c r="F22" s="21"/>
+      <c r="G22" s="21"/>
+      <c r="H22" s="21" t="s">
         <v>21</v>
       </c>
-      <c r="I22" s="9"/>
-      <c r="J22" s="9"/>
-      <c r="K22" s="9"/>
-      <c r="L22" s="9"/>
-      <c r="M22" s="9"/>
-      <c r="N22" s="9"/>
+      <c r="I22" s="21"/>
+      <c r="J22" s="21"/>
+      <c r="K22" s="21"/>
+      <c r="L22" s="21"/>
+      <c r="M22" s="21"/>
+      <c r="N22" s="21"/>
     </row>
     <row r="23" spans="1:14" ht="12" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="14" t="s">
+      <c r="A23" s="20" t="s">
         <v>22</v>
       </c>
-      <c r="B23" s="9"/>
-      <c r="C23" s="9"/>
-      <c r="D23" s="9"/>
-      <c r="E23" s="9"/>
-      <c r="F23" s="9"/>
-      <c r="G23" s="19"/>
-      <c r="H23" s="20"/>
-      <c r="I23" s="20"/>
-      <c r="J23" s="20"/>
-      <c r="K23" s="20"/>
-      <c r="L23" s="20"/>
-      <c r="M23" s="20"/>
-      <c r="N23" s="21"/>
+      <c r="B23" s="21"/>
+      <c r="C23" s="21"/>
+      <c r="D23" s="21"/>
+      <c r="E23" s="21"/>
+      <c r="F23" s="21"/>
+      <c r="G23" s="17"/>
+      <c r="H23" s="18"/>
+      <c r="I23" s="18"/>
+      <c r="J23" s="18"/>
+      <c r="K23" s="18"/>
+      <c r="L23" s="18"/>
+      <c r="M23" s="18"/>
+      <c r="N23" s="19"/>
     </row>
     <row r="24" spans="1:14" ht="22.2" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="14" t="s">
+      <c r="A24" s="20" t="s">
         <v>23</v>
       </c>
-      <c r="B24" s="9"/>
-      <c r="C24" s="9"/>
-      <c r="D24" s="9"/>
-      <c r="E24" s="9"/>
-      <c r="F24" s="9"/>
+      <c r="B24" s="21"/>
+      <c r="C24" s="21"/>
+      <c r="D24" s="21"/>
+      <c r="E24" s="21"/>
+      <c r="F24" s="21"/>
       <c r="G24" s="22" t="s">
         <v>24</v>
       </c>
@@ -1517,13 +1520,13 @@
       <c r="C26" s="7"/>
       <c r="D26" s="7"/>
       <c r="E26" s="7"/>
-      <c r="F26" s="19" t="s">
+      <c r="F26" s="17" t="s">
         <v>27</v>
       </c>
-      <c r="G26" s="20"/>
-      <c r="H26" s="20"/>
-      <c r="I26" s="20"/>
-      <c r="J26" s="21"/>
+      <c r="G26" s="18"/>
+      <c r="H26" s="18"/>
+      <c r="I26" s="18"/>
+      <c r="J26" s="19"/>
       <c r="K26" s="7" t="s">
         <v>28</v>
       </c>
@@ -1535,19 +1538,19 @@
       <c r="A27" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="B27" s="32"/>
-      <c r="C27" s="32"/>
-      <c r="D27" s="32"/>
-      <c r="E27" s="32"/>
-      <c r="F27" s="29"/>
-      <c r="G27" s="30"/>
-      <c r="H27" s="30"/>
-      <c r="I27" s="30"/>
-      <c r="J27" s="31"/>
-      <c r="K27" s="32"/>
-      <c r="L27" s="32"/>
-      <c r="M27" s="32"/>
-      <c r="N27" s="32"/>
+      <c r="B27" s="12"/>
+      <c r="C27" s="12"/>
+      <c r="D27" s="12"/>
+      <c r="E27" s="12"/>
+      <c r="F27" s="8"/>
+      <c r="G27" s="9"/>
+      <c r="H27" s="9"/>
+      <c r="I27" s="9"/>
+      <c r="J27" s="10"/>
+      <c r="K27" s="12"/>
+      <c r="L27" s="12"/>
+      <c r="M27" s="12"/>
+      <c r="N27" s="12"/>
     </row>
     <row r="28" spans="1:14" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="5" t="s">
@@ -1557,54 +1560,81 @@
       <c r="C28" s="7"/>
       <c r="D28" s="7"/>
       <c r="E28" s="7"/>
-      <c r="F28" s="29"/>
-      <c r="G28" s="30"/>
-      <c r="H28" s="30"/>
-      <c r="I28" s="30"/>
-      <c r="J28" s="31"/>
-      <c r="K28" s="33"/>
-      <c r="L28" s="32"/>
-      <c r="M28" s="32"/>
-      <c r="N28" s="32"/>
+      <c r="F28" s="8"/>
+      <c r="G28" s="9"/>
+      <c r="H28" s="9"/>
+      <c r="I28" s="9"/>
+      <c r="J28" s="10"/>
+      <c r="K28" s="11"/>
+      <c r="L28" s="12"/>
+      <c r="M28" s="12"/>
+      <c r="N28" s="12"/>
     </row>
     <row r="29" spans="1:14" ht="16.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="B29" s="34"/>
+      <c r="B29" s="13"/>
       <c r="C29" s="7"/>
       <c r="D29" s="7"/>
       <c r="E29" s="7"/>
-      <c r="F29" s="35"/>
-      <c r="G29" s="36"/>
-      <c r="H29" s="36"/>
-      <c r="I29" s="36"/>
-      <c r="J29" s="37"/>
-      <c r="K29" s="34"/>
+      <c r="F29" s="14"/>
+      <c r="G29" s="15"/>
+      <c r="H29" s="15"/>
+      <c r="I29" s="15"/>
+      <c r="J29" s="16"/>
+      <c r="K29" s="13"/>
       <c r="L29" s="7"/>
       <c r="M29" s="7"/>
       <c r="N29" s="7"/>
     </row>
   </sheetData>
   <mergeCells count="77">
-    <mergeCell ref="B28:E28"/>
-    <mergeCell ref="F28:J28"/>
-    <mergeCell ref="K28:N28"/>
-    <mergeCell ref="B29:E29"/>
-    <mergeCell ref="F29:J29"/>
-    <mergeCell ref="K29:N29"/>
-    <mergeCell ref="A26:E26"/>
-    <mergeCell ref="F26:J26"/>
-    <mergeCell ref="K26:N26"/>
-    <mergeCell ref="B27:E27"/>
-    <mergeCell ref="F27:J27"/>
-    <mergeCell ref="K27:N27"/>
-    <mergeCell ref="A23:F23"/>
-    <mergeCell ref="G23:N23"/>
-    <mergeCell ref="A24:F24"/>
-    <mergeCell ref="G24:N24"/>
-    <mergeCell ref="A25:B25"/>
-    <mergeCell ref="C25:N25"/>
+    <mergeCell ref="A1:B4"/>
+    <mergeCell ref="C1:K4"/>
+    <mergeCell ref="L1:N1"/>
+    <mergeCell ref="L2:N2"/>
+    <mergeCell ref="L3:N3"/>
+    <mergeCell ref="L4:N4"/>
+    <mergeCell ref="A7:A8"/>
+    <mergeCell ref="B7:F8"/>
+    <mergeCell ref="G7:I7"/>
+    <mergeCell ref="J7:J8"/>
+    <mergeCell ref="K7:L7"/>
+    <mergeCell ref="A5:E5"/>
+    <mergeCell ref="F5:K5"/>
+    <mergeCell ref="L5:N5"/>
+    <mergeCell ref="A6:I6"/>
+    <mergeCell ref="J6:N6"/>
+    <mergeCell ref="M7:N8"/>
+    <mergeCell ref="G8:H8"/>
+    <mergeCell ref="B9:F9"/>
+    <mergeCell ref="G9:H9"/>
+    <mergeCell ref="M9:N9"/>
+    <mergeCell ref="B10:F10"/>
+    <mergeCell ref="G10:H10"/>
+    <mergeCell ref="M10:N10"/>
+    <mergeCell ref="B11:F11"/>
+    <mergeCell ref="G11:H11"/>
+    <mergeCell ref="M11:N11"/>
+    <mergeCell ref="B12:F12"/>
+    <mergeCell ref="G12:H12"/>
+    <mergeCell ref="M12:N12"/>
+    <mergeCell ref="B13:F13"/>
+    <mergeCell ref="G13:H13"/>
+    <mergeCell ref="M13:N13"/>
+    <mergeCell ref="B14:F14"/>
+    <mergeCell ref="G14:H14"/>
+    <mergeCell ref="M14:N14"/>
+    <mergeCell ref="B15:F15"/>
+    <mergeCell ref="G15:H15"/>
+    <mergeCell ref="M15:N15"/>
+    <mergeCell ref="B16:F16"/>
+    <mergeCell ref="G16:H16"/>
+    <mergeCell ref="M16:N16"/>
+    <mergeCell ref="B17:F17"/>
+    <mergeCell ref="G17:H17"/>
+    <mergeCell ref="M17:N17"/>
     <mergeCell ref="B18:F18"/>
     <mergeCell ref="G18:H18"/>
     <mergeCell ref="M18:N18"/>
@@ -1619,51 +1649,24 @@
     <mergeCell ref="B21:F21"/>
     <mergeCell ref="G21:H21"/>
     <mergeCell ref="M21:N21"/>
-    <mergeCell ref="B16:F16"/>
-    <mergeCell ref="G16:H16"/>
-    <mergeCell ref="M16:N16"/>
-    <mergeCell ref="B17:F17"/>
-    <mergeCell ref="G17:H17"/>
-    <mergeCell ref="M17:N17"/>
-    <mergeCell ref="B14:F14"/>
-    <mergeCell ref="G14:H14"/>
-    <mergeCell ref="M14:N14"/>
-    <mergeCell ref="B15:F15"/>
-    <mergeCell ref="G15:H15"/>
-    <mergeCell ref="M15:N15"/>
-    <mergeCell ref="B12:F12"/>
-    <mergeCell ref="G12:H12"/>
-    <mergeCell ref="M12:N12"/>
-    <mergeCell ref="B13:F13"/>
-    <mergeCell ref="G13:H13"/>
-    <mergeCell ref="M13:N13"/>
-    <mergeCell ref="B10:F10"/>
-    <mergeCell ref="G10:H10"/>
-    <mergeCell ref="M10:N10"/>
-    <mergeCell ref="B11:F11"/>
-    <mergeCell ref="G11:H11"/>
-    <mergeCell ref="M11:N11"/>
-    <mergeCell ref="M7:N8"/>
-    <mergeCell ref="G8:H8"/>
-    <mergeCell ref="B9:F9"/>
-    <mergeCell ref="G9:H9"/>
-    <mergeCell ref="M9:N9"/>
-    <mergeCell ref="A5:E5"/>
-    <mergeCell ref="F5:K5"/>
-    <mergeCell ref="L5:N5"/>
-    <mergeCell ref="A6:I6"/>
-    <mergeCell ref="J6:N6"/>
-    <mergeCell ref="A7:A8"/>
-    <mergeCell ref="B7:F8"/>
-    <mergeCell ref="G7:I7"/>
-    <mergeCell ref="J7:J8"/>
-    <mergeCell ref="K7:L7"/>
-    <mergeCell ref="A1:B4"/>
-    <mergeCell ref="C1:K4"/>
-    <mergeCell ref="L1:N1"/>
-    <mergeCell ref="L2:N2"/>
-    <mergeCell ref="L3:N3"/>
-    <mergeCell ref="L4:N4"/>
+    <mergeCell ref="A23:F23"/>
+    <mergeCell ref="G23:N23"/>
+    <mergeCell ref="A24:F24"/>
+    <mergeCell ref="G24:N24"/>
+    <mergeCell ref="A25:B25"/>
+    <mergeCell ref="C25:N25"/>
+    <mergeCell ref="A26:E26"/>
+    <mergeCell ref="F26:J26"/>
+    <mergeCell ref="K26:N26"/>
+    <mergeCell ref="B27:E27"/>
+    <mergeCell ref="F27:J27"/>
+    <mergeCell ref="K27:N27"/>
+    <mergeCell ref="B28:E28"/>
+    <mergeCell ref="F28:J28"/>
+    <mergeCell ref="K28:N28"/>
+    <mergeCell ref="B29:E29"/>
+    <mergeCell ref="F29:J29"/>
+    <mergeCell ref="K29:N29"/>
   </mergeCells>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>